<commit_message>
chỉnh text  + template
</commit_message>
<xml_diff>
--- a/portal.solexpress/public/static/etower-create-sample.xlsx
+++ b/portal.solexpress/public/static/etower-create-sample.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="85">
   <si>
     <t>Ref No.</t>
   </si>
@@ -70,9 +70,21 @@
     <t>Shipper Facility/Origin</t>
   </si>
   <si>
+    <t>Return Country</t>
+  </si>
+  <si>
     <t>Return Name</t>
   </si>
   <si>
+    <t>Return State</t>
+  </si>
+  <si>
+    <t>Return Phone</t>
+  </si>
+  <si>
+    <t>Return Postcode</t>
+  </si>
+  <si>
     <t>Shipper Company Name</t>
   </si>
   <si>
@@ -82,6 +94,33 @@
     <t>Shipper Name</t>
   </si>
   <si>
+    <t>Service Option</t>
+  </si>
+  <si>
+    <t>Shipper Organization Code</t>
+  </si>
+  <si>
+    <t>Shipper Email</t>
+  </si>
+  <si>
+    <t>Shipper Postcode</t>
+  </si>
+  <si>
+    <t>Shipper State</t>
+  </si>
+  <si>
+    <t>Shipper City</t>
+  </si>
+  <si>
+    <t>Shipper Address Line 1</t>
+  </si>
+  <si>
+    <t>Shipper Phone</t>
+  </si>
+  <si>
+    <t>Shipper Country</t>
+  </si>
+  <si>
     <t>referenceNo</t>
   </si>
   <si>
@@ -142,12 +181,51 @@
     <t>returnCountry</t>
   </si>
   <si>
+    <t>returnName</t>
+  </si>
+  <si>
+    <t>returnState</t>
+  </si>
+  <si>
+    <t>returnPhone</t>
+  </si>
+  <si>
+    <t>returnPostcode</t>
+  </si>
+  <si>
     <t>shipperCompanyName</t>
   </si>
   <si>
     <t>shipperName</t>
   </si>
   <si>
+    <t>serviceOption</t>
+  </si>
+  <si>
+    <t>shipperOrganizationCode</t>
+  </si>
+  <si>
+    <t>shipperEmail</t>
+  </si>
+  <si>
+    <t>shipperPostcode</t>
+  </si>
+  <si>
+    <t>shipperState</t>
+  </si>
+  <si>
+    <t>shipperCity</t>
+  </si>
+  <si>
+    <t>shipperAddressLine1</t>
+  </si>
+  <si>
+    <t>shipperPhone</t>
+  </si>
+  <si>
+    <t>shipperCountry</t>
+  </si>
+  <si>
     <t>2222199236410011111</t>
   </si>
   <si>
@@ -185,6 +263,9 @@
   </si>
   <si>
     <t>UBI.AU2AU.AUPOST.Y</t>
+  </si>
+  <si>
+    <t>E-Parcel</t>
   </si>
 </sst>
 </file>
@@ -194,7 +275,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d\.m"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -206,12 +287,6 @@
       <sz val="12.0"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12.0"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <sz val="10.0"/>
@@ -229,6 +304,25 @@
       <name val="Times New Roman"/>
     </font>
     <font>
+      <sz val="12.0"/>
+      <color theme="5"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="12.0"/>
+      <color rgb="FFEA4335"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12.0"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -236,15 +330,10 @@
     <font>
       <sz val="12.0"/>
       <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-    </font>
-    <font>
-      <sz val="12.0"/>
-      <color rgb="FF000000"/>
       <name val="PMingLiu"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -255,12 +344,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor rgb="FFFFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -296,36 +379,42 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="1" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="2" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="2" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="2" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="2" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -565,12 +654,18 @@
     <col customWidth="1" min="17" max="17" width="6.75"/>
     <col customWidth="1" min="18" max="18" width="7.38"/>
     <col customWidth="1" min="19" max="19" width="22.88"/>
-    <col customWidth="1" min="20" max="20" width="14.13"/>
-    <col customWidth="1" min="21" max="22" width="24.63"/>
-    <col customWidth="1" min="23" max="23" width="14.75"/>
-    <col customWidth="1" min="25" max="26" width="20.63"/>
-    <col customWidth="1" min="27" max="27" width="21.0"/>
-    <col customWidth="1" min="28" max="28" width="35.13"/>
+    <col customWidth="1" min="20" max="20" width="14.88"/>
+    <col customWidth="1" min="21" max="26" width="24.63"/>
+    <col customWidth="1" min="27" max="27" width="14.75"/>
+    <col customWidth="1" min="28" max="28" width="13.75"/>
+    <col customWidth="1" min="29" max="29" width="24.5"/>
+    <col customWidth="1" min="30" max="30" width="20.63"/>
+    <col customWidth="1" min="31" max="31" width="21.0"/>
+    <col customWidth="1" min="32" max="32" width="35.13"/>
+    <col customWidth="1" min="33" max="33" width="12.0"/>
+    <col customWidth="1" min="34" max="34" width="21.13"/>
+    <col customWidth="1" min="35" max="35" width="13.63"/>
+    <col customWidth="1" min="36" max="36" width="15.5"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
@@ -631,27 +726,57 @@
       <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="2"/>
-      <c r="AC1" s="3"/>
-      <c r="AD1" s="3"/>
-      <c r="AE1" s="3"/>
-      <c r="AF1" s="3"/>
-      <c r="AG1" s="3"/>
-      <c r="AH1" s="3"/>
-      <c r="AI1" s="3"/>
-      <c r="AJ1" s="3"/>
+      <c r="X1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>35</v>
+      </c>
       <c r="AK1" s="3"/>
       <c r="AL1" s="3"/>
       <c r="AM1" s="3"/>
@@ -659,120 +784,163 @@
       <c r="AO1" s="3"/>
       <c r="AP1" s="3"/>
       <c r="AQ1" s="3"/>
+      <c r="AR1" s="3"/>
+      <c r="AS1" s="3"/>
+      <c r="AT1" s="3"/>
+      <c r="AU1" s="3"/>
     </row>
     <row r="2" ht="15.75" hidden="1" customHeight="1">
       <c r="A2" s="4" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="N2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="T2" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="U2" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="V2" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="W2" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="X2" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y2" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z2" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="J2" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="L2" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="O2" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="P2" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q2" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="R2" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="S2" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="T2" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="U2" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="V2" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="W2" s="4" t="s">
-        <v>44</v>
+      <c r="AA2" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="AB2" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="AC2" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="AD2" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="AE2" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF2" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="AG2" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="AH2" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="AI2" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="AJ2" s="7" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>47</v>
+      <c r="A3" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>73</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>48</v>
+        <v>74</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="G3" s="8">
         <v>4077.0</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>50</v>
+        <v>76</v>
       </c>
       <c r="I3" s="8">
         <v>6.140655734E10</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="K3" s="10">
         <v>120.0</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>52</v>
+        <v>78</v>
       </c>
       <c r="M3" s="8">
         <v>11.0</v>
       </c>
       <c r="N3" s="9" t="s">
-        <v>53</v>
+        <v>79</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>54</v>
+        <v>80</v>
       </c>
       <c r="P3" s="8">
         <v>60.0</v>
@@ -784,19 +952,28 @@
         <v>19.0</v>
       </c>
       <c r="S3" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="T3" s="9" t="s">
-        <v>56</v>
+        <v>81</v>
+      </c>
+      <c r="T3" s="11" t="s">
+        <v>76</v>
       </c>
       <c r="U3" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="V3" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="W3" s="9" t="s">
-        <v>56</v>
+        <v>82</v>
+      </c>
+      <c r="V3" s="9"/>
+      <c r="W3" s="9"/>
+      <c r="X3" s="9"/>
+      <c r="Y3" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="Z3" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="AA3" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="AB3" s="12" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
@@ -821,8 +998,12 @@
       <c r="S4" s="9"/>
       <c r="T4" s="9"/>
       <c r="U4" s="9"/>
-      <c r="V4" s="4"/>
+      <c r="V4" s="9"/>
       <c r="W4" s="9"/>
+      <c r="X4" s="9"/>
+      <c r="Y4" s="9"/>
+      <c r="Z4" s="4"/>
+      <c r="AA4" s="9"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="10"/>
@@ -846,8 +1027,12 @@
       <c r="S5" s="9"/>
       <c r="T5" s="9"/>
       <c r="U5" s="9"/>
-      <c r="V5" s="4"/>
+      <c r="V5" s="9"/>
       <c r="W5" s="9"/>
+      <c r="X5" s="9"/>
+      <c r="Y5" s="9"/>
+      <c r="Z5" s="4"/>
+      <c r="AA5" s="9"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="10"/>
@@ -871,8 +1056,12 @@
       <c r="S6" s="9"/>
       <c r="T6" s="9"/>
       <c r="U6" s="9"/>
-      <c r="V6" s="4"/>
+      <c r="V6" s="9"/>
       <c r="W6" s="9"/>
+      <c r="X6" s="9"/>
+      <c r="Y6" s="9"/>
+      <c r="Z6" s="4"/>
+      <c r="AA6" s="9"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="10"/>
@@ -896,8 +1085,12 @@
       <c r="S7" s="9"/>
       <c r="T7" s="9"/>
       <c r="U7" s="9"/>
-      <c r="V7" s="4"/>
+      <c r="V7" s="9"/>
       <c r="W7" s="9"/>
+      <c r="X7" s="9"/>
+      <c r="Y7" s="9"/>
+      <c r="Z7" s="4"/>
+      <c r="AA7" s="9"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="10"/>
@@ -921,8 +1114,12 @@
       <c r="S8" s="9"/>
       <c r="T8" s="9"/>
       <c r="U8" s="9"/>
-      <c r="V8" s="4"/>
+      <c r="V8" s="9"/>
       <c r="W8" s="9"/>
+      <c r="X8" s="9"/>
+      <c r="Y8" s="9"/>
+      <c r="Z8" s="4"/>
+      <c r="AA8" s="9"/>
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="10"/>
@@ -946,8 +1143,12 @@
       <c r="S9" s="9"/>
       <c r="T9" s="9"/>
       <c r="U9" s="9"/>
-      <c r="V9" s="4"/>
+      <c r="V9" s="9"/>
       <c r="W9" s="9"/>
+      <c r="X9" s="9"/>
+      <c r="Y9" s="9"/>
+      <c r="Z9" s="4"/>
+      <c r="AA9" s="9"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="10"/>
@@ -971,8 +1172,12 @@
       <c r="S10" s="9"/>
       <c r="T10" s="9"/>
       <c r="U10" s="9"/>
-      <c r="V10" s="4"/>
+      <c r="V10" s="9"/>
       <c r="W10" s="9"/>
+      <c r="X10" s="9"/>
+      <c r="Y10" s="9"/>
+      <c r="Z10" s="4"/>
+      <c r="AA10" s="9"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="10"/>
@@ -996,8 +1201,12 @@
       <c r="S11" s="9"/>
       <c r="T11" s="9"/>
       <c r="U11" s="9"/>
-      <c r="V11" s="4"/>
+      <c r="V11" s="9"/>
       <c r="W11" s="9"/>
+      <c r="X11" s="9"/>
+      <c r="Y11" s="9"/>
+      <c r="Z11" s="4"/>
+      <c r="AA11" s="9"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="10"/>
@@ -1021,8 +1230,12 @@
       <c r="S12" s="9"/>
       <c r="T12" s="9"/>
       <c r="U12" s="9"/>
-      <c r="V12" s="4"/>
+      <c r="V12" s="9"/>
       <c r="W12" s="9"/>
+      <c r="X12" s="9"/>
+      <c r="Y12" s="9"/>
+      <c r="Z12" s="4"/>
+      <c r="AA12" s="9"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="10"/>
@@ -1046,8 +1259,12 @@
       <c r="S13" s="9"/>
       <c r="T13" s="9"/>
       <c r="U13" s="9"/>
-      <c r="V13" s="4"/>
+      <c r="V13" s="9"/>
       <c r="W13" s="9"/>
+      <c r="X13" s="9"/>
+      <c r="Y13" s="9"/>
+      <c r="Z13" s="4"/>
+      <c r="AA13" s="9"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="10"/>
@@ -1071,8 +1288,12 @@
       <c r="S14" s="9"/>
       <c r="T14" s="9"/>
       <c r="U14" s="9"/>
-      <c r="V14" s="4"/>
+      <c r="V14" s="9"/>
       <c r="W14" s="9"/>
+      <c r="X14" s="9"/>
+      <c r="Y14" s="9"/>
+      <c r="Z14" s="4"/>
+      <c r="AA14" s="9"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="A15" s="10"/>
@@ -1096,8 +1317,12 @@
       <c r="S15" s="9"/>
       <c r="T15" s="9"/>
       <c r="U15" s="9"/>
-      <c r="V15" s="4"/>
+      <c r="V15" s="9"/>
       <c r="W15" s="9"/>
+      <c r="X15" s="9"/>
+      <c r="Y15" s="9"/>
+      <c r="Z15" s="4"/>
+      <c r="AA15" s="9"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="10"/>
@@ -1121,8 +1346,12 @@
       <c r="S16" s="9"/>
       <c r="T16" s="9"/>
       <c r="U16" s="9"/>
-      <c r="V16" s="4"/>
+      <c r="V16" s="9"/>
       <c r="W16" s="9"/>
+      <c r="X16" s="9"/>
+      <c r="Y16" s="9"/>
+      <c r="Z16" s="4"/>
+      <c r="AA16" s="9"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="A17" s="10"/>
@@ -1146,8 +1375,12 @@
       <c r="S17" s="9"/>
       <c r="T17" s="9"/>
       <c r="U17" s="9"/>
-      <c r="V17" s="4"/>
+      <c r="V17" s="9"/>
       <c r="W17" s="9"/>
+      <c r="X17" s="9"/>
+      <c r="Y17" s="9"/>
+      <c r="Z17" s="4"/>
+      <c r="AA17" s="9"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="10"/>
@@ -1171,8 +1404,12 @@
       <c r="S18" s="9"/>
       <c r="T18" s="9"/>
       <c r="U18" s="9"/>
-      <c r="V18" s="4"/>
+      <c r="V18" s="9"/>
       <c r="W18" s="9"/>
+      <c r="X18" s="9"/>
+      <c r="Y18" s="9"/>
+      <c r="Z18" s="4"/>
+      <c r="AA18" s="9"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="10"/>
@@ -1196,8 +1433,12 @@
       <c r="S19" s="9"/>
       <c r="T19" s="9"/>
       <c r="U19" s="9"/>
-      <c r="V19" s="4"/>
+      <c r="V19" s="9"/>
       <c r="W19" s="9"/>
+      <c r="X19" s="9"/>
+      <c r="Y19" s="9"/>
+      <c r="Z19" s="4"/>
+      <c r="AA19" s="9"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="10"/>
@@ -1221,8 +1462,12 @@
       <c r="S20" s="9"/>
       <c r="T20" s="9"/>
       <c r="U20" s="9"/>
-      <c r="V20" s="4"/>
+      <c r="V20" s="9"/>
       <c r="W20" s="9"/>
+      <c r="X20" s="9"/>
+      <c r="Y20" s="9"/>
+      <c r="Z20" s="4"/>
+      <c r="AA20" s="9"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="10"/>
@@ -1246,8 +1491,12 @@
       <c r="S21" s="9"/>
       <c r="T21" s="9"/>
       <c r="U21" s="9"/>
-      <c r="V21" s="4"/>
+      <c r="V21" s="9"/>
       <c r="W21" s="9"/>
+      <c r="X21" s="9"/>
+      <c r="Y21" s="9"/>
+      <c r="Z21" s="4"/>
+      <c r="AA21" s="9"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="10"/>
@@ -1271,8 +1520,12 @@
       <c r="S22" s="9"/>
       <c r="T22" s="9"/>
       <c r="U22" s="9"/>
-      <c r="V22" s="4"/>
+      <c r="V22" s="9"/>
       <c r="W22" s="9"/>
+      <c r="X22" s="9"/>
+      <c r="Y22" s="9"/>
+      <c r="Z22" s="4"/>
+      <c r="AA22" s="9"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="10"/>
@@ -1296,8 +1549,12 @@
       <c r="S23" s="9"/>
       <c r="T23" s="9"/>
       <c r="U23" s="9"/>
-      <c r="V23" s="4"/>
+      <c r="V23" s="9"/>
       <c r="W23" s="9"/>
+      <c r="X23" s="9"/>
+      <c r="Y23" s="9"/>
+      <c r="Z23" s="4"/>
+      <c r="AA23" s="9"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="10"/>
@@ -1321,8 +1578,12 @@
       <c r="S24" s="9"/>
       <c r="T24" s="9"/>
       <c r="U24" s="9"/>
-      <c r="V24" s="4"/>
+      <c r="V24" s="9"/>
       <c r="W24" s="9"/>
+      <c r="X24" s="9"/>
+      <c r="Y24" s="9"/>
+      <c r="Z24" s="4"/>
+      <c r="AA24" s="9"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="10"/>
@@ -1346,8 +1607,12 @@
       <c r="S25" s="9"/>
       <c r="T25" s="9"/>
       <c r="U25" s="9"/>
-      <c r="V25" s="4"/>
+      <c r="V25" s="9"/>
       <c r="W25" s="9"/>
+      <c r="X25" s="9"/>
+      <c r="Y25" s="9"/>
+      <c r="Z25" s="4"/>
+      <c r="AA25" s="9"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="10"/>
@@ -1362,7 +1627,7 @@
       <c r="J26" s="9"/>
       <c r="K26" s="10"/>
       <c r="L26" s="9"/>
-      <c r="M26" s="11"/>
+      <c r="M26" s="13"/>
       <c r="N26" s="9"/>
       <c r="O26" s="9"/>
       <c r="P26" s="10"/>
@@ -1371,8 +1636,12 @@
       <c r="S26" s="9"/>
       <c r="T26" s="9"/>
       <c r="U26" s="9"/>
-      <c r="V26" s="4"/>
+      <c r="V26" s="9"/>
       <c r="W26" s="9"/>
+      <c r="X26" s="9"/>
+      <c r="Y26" s="9"/>
+      <c r="Z26" s="4"/>
+      <c r="AA26" s="9"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="10"/>
@@ -1396,8 +1665,12 @@
       <c r="S27" s="9"/>
       <c r="T27" s="9"/>
       <c r="U27" s="9"/>
-      <c r="V27" s="4"/>
+      <c r="V27" s="9"/>
       <c r="W27" s="9"/>
+      <c r="X27" s="9"/>
+      <c r="Y27" s="9"/>
+      <c r="Z27" s="4"/>
+      <c r="AA27" s="9"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="10"/>
@@ -1421,8 +1694,12 @@
       <c r="S28" s="9"/>
       <c r="T28" s="9"/>
       <c r="U28" s="9"/>
-      <c r="V28" s="4"/>
+      <c r="V28" s="9"/>
       <c r="W28" s="9"/>
+      <c r="X28" s="9"/>
+      <c r="Y28" s="9"/>
+      <c r="Z28" s="4"/>
+      <c r="AA28" s="9"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="10"/>
@@ -1446,8 +1723,12 @@
       <c r="S29" s="9"/>
       <c r="T29" s="9"/>
       <c r="U29" s="9"/>
-      <c r="V29" s="4"/>
+      <c r="V29" s="9"/>
       <c r="W29" s="9"/>
+      <c r="X29" s="9"/>
+      <c r="Y29" s="9"/>
+      <c r="Z29" s="4"/>
+      <c r="AA29" s="9"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="10"/>
@@ -1471,8 +1752,12 @@
       <c r="S30" s="9"/>
       <c r="T30" s="9"/>
       <c r="U30" s="9"/>
-      <c r="V30" s="4"/>
+      <c r="V30" s="9"/>
       <c r="W30" s="9"/>
+      <c r="X30" s="9"/>
+      <c r="Y30" s="9"/>
+      <c r="Z30" s="4"/>
+      <c r="AA30" s="9"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="10"/>
@@ -1496,11 +1781,15 @@
       <c r="S31" s="9"/>
       <c r="T31" s="9"/>
       <c r="U31" s="9"/>
-      <c r="V31" s="4"/>
+      <c r="V31" s="9"/>
       <c r="W31" s="9"/>
+      <c r="X31" s="9"/>
+      <c r="Y31" s="9"/>
+      <c r="Z31" s="4"/>
+      <c r="AA31" s="9"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="S32" s="12"/>
+      <c r="S32" s="14"/>
     </row>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="15.75" customHeight="1"/>
@@ -2468,6 +2757,8 @@
     <row r="996" ht="15.75" customHeight="1"/>
     <row r="997" ht="15.75" customHeight="1"/>
     <row r="998" ht="15.75" customHeight="1"/>
+    <row r="999" ht="15.75" customHeight="1"/>
+    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>